<commit_message>
Updated graph titles and labels
</commit_message>
<xml_diff>
--- a/pandemic-loss-modeling/exceedance_results/bernstein_original.xlsx
+++ b/pandemic-loss-modeling/exceedance_results/bernstein_original.xlsx
@@ -377,7 +377,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -470,145 +470,177 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B12">
-        <v>0.005337135165461502</v>
+        <v>0.006708732254968096</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="B13">
-        <v>0.001851572823087372</v>
+        <v>0.005337135165461502</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="B14">
-        <v>0.001282168873004006</v>
+        <v>0.003519466328820613</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="B15">
-        <v>0.001135589253560032</v>
+        <v>0.002618054326933769</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16">
-        <v>70</v>
+        <v>28</v>
       </c>
       <c r="B16">
-        <v>0.0007200633024848703</v>
+        <v>0.001851572823087372</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17">
-        <v>86</v>
+        <v>40</v>
       </c>
       <c r="B17">
-        <v>0.000582319971139508</v>
+        <v>0.001282168873004006</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18">
-        <v>100</v>
+        <v>45</v>
       </c>
       <c r="B18">
-        <v>0.0004984175336785841</v>
+        <v>0.001135589253560032</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19">
-        <v>120</v>
+        <v>70</v>
       </c>
       <c r="B19">
-        <v>0.000412957220595775</v>
+        <v>0.0007200633024848703</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20">
-        <v>150</v>
+        <v>86</v>
       </c>
       <c r="B20">
-        <v>0.0003280319599882583</v>
+        <v>0.000582319971139508</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21">
-        <v>170</v>
+        <v>100</v>
       </c>
       <c r="B21">
-        <v>0.000288288457553622</v>
+        <v>0.0004984175336785841</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22">
-        <v>190</v>
+        <v>120</v>
       </c>
       <c r="B22">
-        <v>0.0002570288724353808</v>
+        <v>0.000412957220595775</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="B23">
-        <v>0.0002437779286262874</v>
+        <v>0.0003280319599882583</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24">
-        <v>220</v>
+        <v>170</v>
       </c>
       <c r="B24">
-        <v>0.0002209425359856459</v>
+        <v>0.000288288457553622</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25">
-        <v>240</v>
+        <v>190</v>
       </c>
       <c r="B25">
-        <v>0.0002019679817690056</v>
+        <v>0.0002570288724353808</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="B26">
-        <v>0.0001936362162571785</v>
+        <v>0.0002437779286262874</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27">
-        <v>260</v>
+        <v>220</v>
       </c>
       <c r="B27">
-        <v>0.0001859551228667904</v>
+        <v>0.0002209425359856459</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28">
-        <v>270</v>
+        <v>230</v>
       </c>
       <c r="B28">
-        <v>0.0001788516891796067</v>
+        <v>0.0002110362371906505</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29">
+        <v>240</v>
+      </c>
+      <c r="B29">
+        <v>0.0002019679817690056</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30">
+        <v>250</v>
+      </c>
+      <c r="B30">
+        <v>0.0001936362162571785</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31">
+        <v>260</v>
+      </c>
+      <c r="B31">
+        <v>0.0001859551228667904</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="A32">
+        <v>270</v>
+      </c>
+      <c r="B32">
+        <v>0.0001788516891796067</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33">
         <v>280</v>
       </c>
-      <c r="B29">
+      <c r="B33">
         <v>0.0001722634086180085</v>
       </c>
     </row>

</xml_diff>